<commit_message>
fixed error in stim_group_lists_tests for groups 6 and 7
groups 6 and 7 had some incorrect non-native learned words listed
</commit_message>
<xml_diff>
--- a/stim/stim_group_lists_test.xlsx
+++ b/stim/stim_group_lists_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\speechres\Task_SpeechMotorSequenceLearning\stim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3077E668-69D0-4B87-97B9-7FA3DD37D122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBBB3982-7C1D-4066-8E92-C62AE53EDAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -552,10 +552,10 @@
         <v>9</v>
       </c>
       <c r="F2" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>2</v>
@@ -584,10 +584,10 @@
         <v>9</v>
       </c>
       <c r="F3" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G3" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>2</v>
@@ -616,10 +616,10 @@
         <v>9</v>
       </c>
       <c r="F4" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G4" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>2</v>
@@ -648,10 +648,10 @@
         <v>9</v>
       </c>
       <c r="F5" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G5" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>2</v>
@@ -680,7 +680,7 @@
         <v>9</v>
       </c>
       <c r="F6" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G6" s="1">
         <v>13</v>
@@ -712,7 +712,7 @@
         <v>9</v>
       </c>
       <c r="F7" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G7" s="1">
         <v>13</v>
@@ -744,7 +744,7 @@
         <v>10</v>
       </c>
       <c r="F8" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="1">
         <v>14</v>
@@ -776,7 +776,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G9" s="1">
         <v>14</v>
@@ -808,7 +808,7 @@
         <v>10</v>
       </c>
       <c r="F10" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G10" s="1">
         <v>14</v>
@@ -840,7 +840,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G11" s="1">
         <v>14</v>
@@ -872,7 +872,7 @@
         <v>10</v>
       </c>
       <c r="F12" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G12" s="1">
         <v>14</v>
@@ -904,7 +904,7 @@
         <v>10</v>
       </c>
       <c r="F13" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G13" s="1">
         <v>14</v>

</xml_diff>

<commit_message>
made Testing phase natives identical to Training phase natives
-changed the stim list for the Testing phase so that it now uses the same native clusters as are used during Training; this means that during testing, we use "learned native" instead of "novel native" clusters
-the natives containing the same coda as non-natives (**UB) are no longer used
</commit_message>
<xml_diff>
--- a/stim/stim_group_lists_test.xlsx
+++ b/stim/stim_group_lists_test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\speechres\Task_SpeechMotorSequenceLearning\stim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amsme\OneDrive\Documents\code\matlab\Task_SpeechMotorSequenceLearning\stim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBBB3982-7C1D-4066-8E92-C62AE53EDAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3905B148-91D0-4270-BB03-360400C778DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="34">
   <si>
-    <t>native</t>
-  </si>
-  <si>
     <t>non-native novel</t>
   </si>
   <si>
@@ -69,18 +66,6 @@
     <t>STOP (non-native novel)</t>
   </si>
   <si>
-    <t>37, 41, 45</t>
-  </si>
-  <si>
-    <t>38, 42, 46</t>
-  </si>
-  <si>
-    <t>39, 43, 47</t>
-  </si>
-  <si>
-    <t>40, 44, 48</t>
-  </si>
-  <si>
     <t>group6</t>
   </si>
   <si>
@@ -127,6 +112,21 @@
   </si>
   <si>
     <t>2, 4, 6</t>
+  </si>
+  <si>
+    <t>native learned</t>
+  </si>
+  <si>
+    <t>25, 29, 35</t>
+  </si>
+  <si>
+    <t>26, 30, 34</t>
+  </si>
+  <si>
+    <t>27, 31, 33</t>
+  </si>
+  <si>
+    <t>28, 32, 36</t>
   </si>
 </sst>
 </file>
@@ -505,34 +505,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -558,7 +558,7 @@
         <v>13</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2" s="1">
         <v>1</v>
@@ -590,7 +590,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" s="1">
         <v>1</v>
@@ -622,7 +622,7 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="1">
         <v>1</v>
@@ -654,7 +654,7 @@
         <v>13</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="1">
         <v>1</v>
@@ -686,7 +686,7 @@
         <v>13</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="1">
         <v>1</v>
@@ -718,7 +718,7 @@
         <v>13</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="1">
         <v>1</v>
@@ -750,7 +750,7 @@
         <v>14</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" s="1">
         <v>1</v>
@@ -782,7 +782,7 @@
         <v>14</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" s="1">
         <v>1</v>
@@ -814,7 +814,7 @@
         <v>14</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="1">
         <v>1</v>
@@ -846,7 +846,7 @@
         <v>14</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I11" s="1">
         <v>1</v>
@@ -878,7 +878,7 @@
         <v>14</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" s="1">
         <v>1</v>
@@ -910,7 +910,7 @@
         <v>14</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" s="1">
         <v>1</v>
@@ -942,7 +942,7 @@
         <v>1</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" s="1">
         <v>2</v>
@@ -974,7 +974,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="1">
         <v>2</v>
@@ -1006,7 +1006,7 @@
         <v>3</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16" s="1">
         <v>2</v>
@@ -1038,7 +1038,7 @@
         <v>4</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" s="1">
         <v>2</v>
@@ -1070,7 +1070,7 @@
         <v>5</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" s="1">
         <v>2</v>
@@ -1102,7 +1102,7 @@
         <v>6</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="1">
         <v>2</v>
@@ -1134,7 +1134,7 @@
         <v>7</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" s="1">
         <v>2</v>
@@ -1166,7 +1166,7 @@
         <v>8</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" s="1">
         <v>2</v>
@@ -1198,7 +1198,7 @@
         <v>9</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" s="1">
         <v>2</v>
@@ -1230,7 +1230,7 @@
         <v>10</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23" s="1">
         <v>2</v>
@@ -1262,7 +1262,7 @@
         <v>11</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I24" s="1">
         <v>2</v>
@@ -1294,7 +1294,7 @@
         <v>12</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" s="1">
         <v>2</v>
@@ -1304,29 +1304,29 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="4">
-        <v>37</v>
+      <c r="A26" s="1">
+        <v>25</v>
       </c>
       <c r="B26" s="1">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="C26" s="1">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D26" s="1">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E26" s="1">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F26" s="1">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G26" s="1">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I26" s="1">
         <v>3</v>
@@ -1336,29 +1336,29 @@
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="4">
-        <v>38</v>
+      <c r="A27" s="1">
+        <v>26</v>
       </c>
       <c r="B27" s="1">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C27" s="1">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="D27" s="1">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E27" s="1">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="F27" s="1">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G27" s="1">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I27" s="1">
         <v>3</v>
@@ -1368,29 +1368,29 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="4">
-        <v>39</v>
+      <c r="A28" s="1">
+        <v>27</v>
       </c>
       <c r="B28" s="1">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C28" s="1">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D28" s="1">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E28" s="1">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="F28" s="1">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G28" s="1">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I28" s="1">
         <v>3</v>
@@ -1400,29 +1400,29 @@
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="4">
-        <v>40</v>
+      <c r="A29" s="1">
+        <v>28</v>
       </c>
       <c r="B29" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="C29" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D29" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E29" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="F29" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G29" s="1">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I29" s="1">
         <v>3</v>
@@ -1432,29 +1432,29 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="4">
-        <v>41</v>
+      <c r="A30" s="1">
+        <v>29</v>
       </c>
       <c r="B30" s="1">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C30" s="1">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D30" s="1">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="E30" s="1">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F30" s="1">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G30" s="1">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I30" s="1">
         <v>3</v>
@@ -1464,29 +1464,29 @@
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="4">
-        <v>42</v>
+      <c r="A31" s="1">
+        <v>30</v>
       </c>
       <c r="B31" s="1">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C31" s="1">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D31" s="1">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="E31" s="1">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F31" s="1">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G31" s="1">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I31" s="1">
         <v>3</v>
@@ -1496,29 +1496,29 @@
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="4">
-        <v>43</v>
+      <c r="A32" s="1">
+        <v>31</v>
       </c>
       <c r="B32" s="1">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C32" s="1">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D32" s="1">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="E32" s="1">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="F32" s="1">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="G32" s="1">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I32" s="1">
         <v>3</v>
@@ -1528,29 +1528,29 @@
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" s="4">
-        <v>44</v>
+      <c r="A33" s="1">
+        <v>32</v>
       </c>
       <c r="B33" s="1">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C33" s="1">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="D33" s="1">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="E33" s="1">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="F33" s="1">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G33" s="1">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I33" s="1">
         <v>3</v>
@@ -1560,29 +1560,29 @@
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" s="4">
-        <v>45</v>
+      <c r="A34" s="1">
+        <v>33</v>
       </c>
       <c r="B34" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C34" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D34" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E34" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="F34" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G34" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I34" s="1">
         <v>3</v>
@@ -1592,29 +1592,29 @@
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="4">
-        <v>46</v>
+      <c r="A35" s="1">
+        <v>34</v>
       </c>
       <c r="B35" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C35" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D35" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E35" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="F35" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G35" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I35" s="1">
         <v>3</v>
@@ -1624,29 +1624,29 @@
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A36" s="4">
-        <v>47</v>
+      <c r="A36" s="1">
+        <v>35</v>
       </c>
       <c r="B36" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="C36" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D36" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E36" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="F36" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G36" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I36" s="1">
         <v>3</v>
@@ -1656,29 +1656,29 @@
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A37" s="4">
-        <v>48</v>
+      <c r="A37" s="1">
+        <v>36</v>
       </c>
       <c r="B37" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C37" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="D37" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E37" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="F37" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="G37" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I37" s="1">
         <v>3</v>
@@ -1710,7 +1710,7 @@
         <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I38" s="1">
         <v>1</v>
@@ -1742,7 +1742,7 @@
         <v>13</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I39" s="1">
         <v>1</v>
@@ -1774,7 +1774,7 @@
         <v>14</v>
       </c>
       <c r="H40" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I40" s="1">
         <v>1</v>
@@ -1806,7 +1806,7 @@
         <v>14</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I41" s="1">
         <v>1</v>
@@ -1817,28 +1817,28 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E42" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C42" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="F42" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H42" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I42" s="1">
         <v>2</v>
@@ -1849,28 +1849,28 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F43" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="H43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I43" s="1">
         <v>2</v>
@@ -1881,28 +1881,28 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="H44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I44" s="1">
         <v>2</v>
@@ -1913,156 +1913,156 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="C45" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="E45" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H45" t="s">
+        <v>12</v>
+      </c>
+      <c r="I45" s="1">
+        <v>2</v>
+      </c>
+      <c r="J45" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>30</v>
+      </c>
+      <c r="B46" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" t="s">
+        <v>30</v>
+      </c>
+      <c r="D46" t="s">
+        <v>30</v>
+      </c>
+      <c r="E46" t="s">
+        <v>30</v>
+      </c>
+      <c r="F46" t="s">
+        <v>30</v>
+      </c>
+      <c r="G46" t="s">
+        <v>30</v>
+      </c>
+      <c r="H46" t="s">
+        <v>11</v>
+      </c>
+      <c r="I46" s="1">
+        <v>3</v>
+      </c>
+      <c r="J46" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>31</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="B47" t="s">
+        <v>31</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47" t="s">
+        <v>31</v>
+      </c>
+      <c r="E47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F47" t="s">
+        <v>31</v>
+      </c>
+      <c r="G47" t="s">
+        <v>31</v>
+      </c>
+      <c r="H47" t="s">
+        <v>11</v>
+      </c>
+      <c r="I47" s="1">
+        <v>3</v>
+      </c>
+      <c r="J47" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" t="s">
+        <v>32</v>
+      </c>
+      <c r="C48" t="s">
+        <v>32</v>
+      </c>
+      <c r="D48" t="s">
+        <v>32</v>
+      </c>
+      <c r="E48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48" t="s">
+        <v>32</v>
+      </c>
+      <c r="G48" t="s">
+        <v>32</v>
+      </c>
+      <c r="H48" t="s">
+        <v>11</v>
+      </c>
+      <c r="I48" s="1">
+        <v>3</v>
+      </c>
+      <c r="J48" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>33</v>
       </c>
-      <c r="E45" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H45" t="s">
-        <v>13</v>
-      </c>
-      <c r="I45" s="1">
-        <v>2</v>
-      </c>
-      <c r="J45" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H46" t="s">
-        <v>12</v>
-      </c>
-      <c r="I46" s="1">
-        <v>3</v>
-      </c>
-      <c r="J46" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H47" t="s">
-        <v>12</v>
-      </c>
-      <c r="I47" s="1">
-        <v>3</v>
-      </c>
-      <c r="J47" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H48" t="s">
-        <v>12</v>
-      </c>
-      <c r="I48" s="1">
-        <v>3</v>
-      </c>
-      <c r="J48" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>17</v>
+      <c r="B49" t="s">
+        <v>33</v>
+      </c>
+      <c r="C49" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49" t="s">
+        <v>33</v>
+      </c>
+      <c r="E49" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" t="s">
+        <v>33</v>
       </c>
       <c r="H49" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I49" s="1">
         <v>3</v>

</xml_diff>